<commit_message>
fixed typo in data
</commit_message>
<xml_diff>
--- a/publications/data.xlsx
+++ b/publications/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/91720c579d88d817/Documents/GitHub/rjjanse.github.io/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="336" documentId="8_{73F58B86-8A8C-44D2-97E6-524D5F699074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CF3B843-3386-4722-BAC7-F958B0960E37}"/>
+  <xr:revisionPtr revIDLastSave="337" documentId="8_{73F58B86-8A8C-44D2-97E6-524D5F699074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2777A451-A596-4671-A46C-1E006DF020BE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0D0B8934-B9C8-41E7-88BE-115311452A91}"/>
   </bookViews>
@@ -263,9 +263,6 @@
     <t>Retrieval practice using VSAQs vs. MCQs</t>
   </si>
   <si>
-    <t>On machine learning for prediction modellign</t>
-  </si>
-  <si>
     <t>Cardiometabolic proteins and kidney function</t>
   </si>
   <si>
@@ -858,6 +855,9 @@
   </si>
   <si>
     <t>pfd_neph</t>
+  </si>
+  <si>
+    <t>On machine learning for prediction modelling</t>
   </si>
 </sst>
 </file>
@@ -1268,7 +1268,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1289,7 +1289,7 @@
         <v>8</v>
       </c>
       <c r="K1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="L1" t="s">
         <v>9</v>
@@ -1322,7 +1322,7 @@
         <v>18</v>
       </c>
       <c r="V1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
@@ -1366,25 +1366,25 @@
         <v>0</v>
       </c>
       <c r="N2" t="s">
+        <v>78</v>
+      </c>
+      <c r="O2" t="s">
         <v>79</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>80</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>81</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="V2" t="b">
         <v>0</v>
@@ -1431,28 +1431,28 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
+        <v>86</v>
+      </c>
+      <c r="O3" t="s">
+        <v>85</v>
+      </c>
+      <c r="P3" t="s">
         <v>87</v>
       </c>
-      <c r="O3" t="s">
-        <v>86</v>
-      </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>88</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="T3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="U3" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="V3" t="b">
         <v>0</v>
@@ -1499,25 +1499,25 @@
         <v>0</v>
       </c>
       <c r="N4" t="s">
+        <v>93</v>
+      </c>
+      <c r="O4" t="s">
         <v>94</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>95</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>96</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="V4" t="b">
         <v>0</v>
@@ -1564,28 +1564,28 @@
         <v>0</v>
       </c>
       <c r="N5" t="s">
+        <v>100</v>
+      </c>
+      <c r="O5" t="s">
         <v>101</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>102</v>
       </c>
-      <c r="P5" t="s">
-        <v>103</v>
-      </c>
       <c r="Q5" t="s">
+        <v>106</v>
+      </c>
+      <c r="R5" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="S5" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="T5" s="1" t="s">
+      <c r="U5" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="V5" t="b">
         <v>0</v>
@@ -1632,28 +1632,28 @@
         <v>0</v>
       </c>
       <c r="N6" t="s">
+        <v>103</v>
+      </c>
+      <c r="O6" t="s">
         <v>104</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>105</v>
       </c>
-      <c r="P6" t="s">
-        <v>106</v>
-      </c>
       <c r="Q6" t="s">
+        <v>111</v>
+      </c>
+      <c r="R6" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="R6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="T6" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="T6" s="1" t="s">
+      <c r="U6" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="V6" t="b">
         <v>0</v>
@@ -1700,25 +1700,25 @@
         <v>1</v>
       </c>
       <c r="N7" t="s">
+        <v>116</v>
+      </c>
+      <c r="O7" t="s">
         <v>117</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>118</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>119</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="R7" s="1" t="s">
+      <c r="S7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="S7" s="1" t="s">
+      <c r="T7" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="V7" t="b">
         <v>0</v>
@@ -1765,25 +1765,25 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
+        <v>123</v>
+      </c>
+      <c r="O8" t="s">
         <v>124</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>125</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>126</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="R8" s="1" t="s">
+      <c r="S8" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="T8" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="V8" t="b">
         <v>0</v>
@@ -1830,28 +1830,28 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
+        <v>130</v>
+      </c>
+      <c r="O9" t="s">
         <v>131</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>132</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>133</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="R9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="T9" s="1" t="s">
+      <c r="U9" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="V9" t="b">
         <v>0</v>
@@ -1898,25 +1898,25 @@
         <v>0</v>
       </c>
       <c r="N10" t="s">
+        <v>138</v>
+      </c>
+      <c r="O10" t="s">
         <v>139</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>140</v>
       </c>
-      <c r="P10" t="s">
-        <v>141</v>
-      </c>
       <c r="Q10" t="s">
+        <v>145</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="R10" s="1" t="s">
+      <c r="S10" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="T10" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="V10" t="b">
         <v>0</v>
@@ -1963,28 +1963,28 @@
         <v>1</v>
       </c>
       <c r="N11" t="s">
+        <v>141</v>
+      </c>
+      <c r="O11" t="s">
         <v>142</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>143</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>144</v>
       </c>
-      <c r="Q11" t="s">
-        <v>145</v>
-      </c>
       <c r="R11" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="S11" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="S11" s="3" t="s">
+      <c r="T11" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="T11" s="3" t="s">
+      <c r="U11" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="U11" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="V11" t="b">
         <v>1</v>
@@ -2096,28 +2096,28 @@
         <v>0</v>
       </c>
       <c r="N13" t="s">
+        <v>254</v>
+      </c>
+      <c r="O13" t="s">
         <v>255</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
+        <v>261</v>
+      </c>
+      <c r="Q13" t="s">
         <v>256</v>
       </c>
-      <c r="P13" t="s">
-        <v>262</v>
-      </c>
-      <c r="Q13" t="s">
+      <c r="R13" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="R13" s="1" t="s">
+      <c r="S13" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="S13" s="1" t="s">
+      <c r="T13" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="T13" s="1" t="s">
+      <c r="U13" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>261</v>
       </c>
       <c r="V13" t="b">
         <v>1</v>
@@ -2164,25 +2164,25 @@
         <v>0</v>
       </c>
       <c r="N14" t="s">
+        <v>247</v>
+      </c>
+      <c r="O14" t="s">
         <v>248</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q14" t="s">
         <v>249</v>
       </c>
-      <c r="P14" t="s">
-        <v>254</v>
-      </c>
-      <c r="Q14" t="s">
+      <c r="R14" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="R14" s="1" t="s">
+      <c r="S14" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="S14" s="1" t="s">
+      <c r="T14" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>253</v>
       </c>
       <c r="V14" t="b">
         <v>0</v>
@@ -2229,25 +2229,25 @@
         <v>1</v>
       </c>
       <c r="N15" t="s">
+        <v>240</v>
+      </c>
+      <c r="O15" t="s">
         <v>241</v>
       </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q15" t="s">
         <v>242</v>
       </c>
-      <c r="P15" t="s">
+      <c r="R15" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="S15" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>243</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="V15" t="b">
         <v>0</v>
@@ -2294,25 +2294,25 @@
         <v>0</v>
       </c>
       <c r="N16" t="s">
+        <v>233</v>
+      </c>
+      <c r="O16" t="s">
         <v>234</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q16" t="s">
         <v>235</v>
       </c>
-      <c r="P16" t="s">
-        <v>240</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="R16" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="R16" s="1" t="s">
+      <c r="S16" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="S16" s="1" t="s">
+      <c r="T16" s="1" t="s">
         <v>238</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>239</v>
       </c>
       <c r="V16" t="b">
         <v>0</v>
@@ -2359,25 +2359,25 @@
         <v>1</v>
       </c>
       <c r="N17" t="s">
+        <v>226</v>
+      </c>
+      <c r="O17" t="s">
         <v>227</v>
       </c>
-      <c r="O17" t="s">
+      <c r="P17" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q17" t="s">
         <v>228</v>
       </c>
-      <c r="P17" t="s">
-        <v>233</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="R17" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="R17" s="1" t="s">
+      <c r="S17" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="T17" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="V17" t="b">
         <v>0</v>
@@ -2424,25 +2424,25 @@
         <v>1</v>
       </c>
       <c r="N18" t="s">
+        <v>219</v>
+      </c>
+      <c r="O18" t="s">
         <v>220</v>
       </c>
-      <c r="O18" t="s">
+      <c r="P18" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q18" t="s">
         <v>221</v>
       </c>
-      <c r="P18" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q18" t="s">
+      <c r="R18" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="R18" s="1" t="s">
+      <c r="S18" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="S18" s="1" t="s">
+      <c r="T18" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>225</v>
       </c>
       <c r="V18" t="b">
         <v>0</v>
@@ -2489,28 +2489,28 @@
         <v>0</v>
       </c>
       <c r="N19" t="s">
+        <v>211</v>
+      </c>
+      <c r="O19" t="s">
         <v>212</v>
       </c>
-      <c r="O19" t="s">
+      <c r="P19" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q19" t="s">
         <v>213</v>
       </c>
-      <c r="P19" t="s">
-        <v>219</v>
-      </c>
-      <c r="Q19" t="s">
+      <c r="R19" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="R19" s="1" t="s">
+      <c r="S19" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="S19" s="1" t="s">
+      <c r="T19" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="T19" s="1" t="s">
+      <c r="U19" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="V19" t="b">
         <v>0</v>
@@ -2557,25 +2557,25 @@
         <v>0</v>
       </c>
       <c r="N20" t="s">
+        <v>204</v>
+      </c>
+      <c r="O20" t="s">
         <v>205</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q20" t="s">
         <v>206</v>
       </c>
-      <c r="P20" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q20" t="s">
+      <c r="R20" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="R20" s="1" t="s">
+      <c r="S20" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="S20" s="1" t="s">
+      <c r="T20" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="V20" t="b">
         <v>0</v>
@@ -2586,7 +2586,7 @@
         <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C21" t="b">
         <v>0</v>
@@ -2622,25 +2622,25 @@
         <v>0</v>
       </c>
       <c r="N21" t="s">
+        <v>197</v>
+      </c>
+      <c r="O21" t="s">
         <v>198</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q21" t="s">
         <v>199</v>
       </c>
-      <c r="P21" t="s">
-        <v>204</v>
-      </c>
-      <c r="Q21" t="s">
+      <c r="R21" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="R21" s="1" t="s">
+      <c r="S21" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="S21" s="1" t="s">
+      <c r="T21" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="V21" t="b">
         <v>0</v>
@@ -2687,25 +2687,25 @@
         <v>0</v>
       </c>
       <c r="N22" t="s">
+        <v>190</v>
+      </c>
+      <c r="O22" t="s">
         <v>191</v>
       </c>
-      <c r="O22" t="s">
+      <c r="P22" t="s">
         <v>192</v>
       </c>
-      <c r="P22" t="s">
+      <c r="Q22" t="s">
         <v>193</v>
       </c>
-      <c r="Q22" t="s">
+      <c r="R22" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="R22" s="1" t="s">
+      <c r="S22" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="S22" s="1" t="s">
+      <c r="T22" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="V22" t="b">
         <v>0</v>
@@ -2752,25 +2752,25 @@
         <v>0</v>
       </c>
       <c r="N23" t="s">
+        <v>183</v>
+      </c>
+      <c r="O23" t="s">
         <v>184</v>
       </c>
-      <c r="O23" t="s">
+      <c r="P23" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q23" t="s">
         <v>185</v>
       </c>
-      <c r="P23" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q23" t="s">
+      <c r="R23" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="S23" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="R23" s="1" t="s">
+      <c r="T23" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="V23" t="b">
         <v>0</v>
@@ -2817,25 +2817,25 @@
         <v>1</v>
       </c>
       <c r="N24" t="s">
+        <v>176</v>
+      </c>
+      <c r="O24" t="s">
         <v>177</v>
       </c>
-      <c r="O24" t="s">
+      <c r="P24" t="s">
         <v>178</v>
       </c>
-      <c r="P24" t="s">
+      <c r="Q24" t="s">
+        <v>180</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="Q24" t="s">
+      <c r="S24" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="R24" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="S24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>183</v>
       </c>
       <c r="V24" t="b">
         <v>0</v>
@@ -2846,7 +2846,7 @@
         <v>67</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>273</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
@@ -2882,28 +2882,28 @@
         <v>0</v>
       </c>
       <c r="N25" t="s">
+        <v>168</v>
+      </c>
+      <c r="O25" t="s">
         <v>169</v>
       </c>
-      <c r="O25" t="s">
+      <c r="P25" t="s">
         <v>170</v>
       </c>
-      <c r="P25" t="s">
+      <c r="Q25" t="s">
         <v>171</v>
       </c>
-      <c r="Q25" t="s">
+      <c r="R25" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="R25" s="1" t="s">
+      <c r="S25" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="S25" s="1" t="s">
+      <c r="T25" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="T25" s="1" t="s">
+      <c r="U25" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="V25" t="b">
         <v>0</v>
@@ -2914,7 +2914,7 @@
         <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="b">
         <v>0</v>
@@ -2950,25 +2950,25 @@
         <v>0</v>
       </c>
       <c r="N26" t="s">
+        <v>161</v>
+      </c>
+      <c r="O26" t="s">
         <v>162</v>
       </c>
-      <c r="O26" t="s">
+      <c r="P26" t="s">
         <v>163</v>
       </c>
-      <c r="P26" t="s">
+      <c r="Q26" t="s">
         <v>164</v>
       </c>
-      <c r="Q26" t="s">
+      <c r="R26" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="R26" s="1" t="s">
+      <c r="S26" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="S26" s="1" t="s">
+      <c r="T26" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="T26" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="V26" t="b">
         <v>0</v>
@@ -2979,7 +2979,7 @@
         <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C27" t="b">
         <v>1</v>
@@ -3015,28 +3015,28 @@
         <v>0</v>
       </c>
       <c r="N27" t="s">
+        <v>154</v>
+      </c>
+      <c r="O27" t="s">
+        <v>264</v>
+      </c>
+      <c r="P27" t="s">
         <v>155</v>
       </c>
-      <c r="O27" t="s">
-        <v>265</v>
-      </c>
-      <c r="P27" t="s">
+      <c r="Q27" t="s">
         <v>156</v>
       </c>
-      <c r="Q27" t="s">
+      <c r="R27" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="R27" s="1" t="s">
+      <c r="S27" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="S27" s="1" t="s">
+      <c r="T27" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="T27" s="1" t="s">
+      <c r="U27" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="U27" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="V27" t="b">
         <v>0</v>
@@ -3047,7 +3047,7 @@
         <v>70</v>
       </c>
       <c r="B28" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C28" t="b">
         <v>0</v>
@@ -3083,25 +3083,25 @@
         <v>0</v>
       </c>
       <c r="N28" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O28" t="s">
+        <v>265</v>
+      </c>
+      <c r="P28" t="s">
         <v>266</v>
       </c>
-      <c r="P28" t="s">
+      <c r="Q28" t="s">
         <v>267</v>
       </c>
-      <c r="Q28" t="s">
+      <c r="R28" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="R28" s="1" t="s">
+      <c r="S28" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="S28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>271</v>
       </c>
       <c r="V28" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
fix error in pfa
</commit_message>
<xml_diff>
--- a/publications/data.xlsx
+++ b/publications/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umcutrecht-my.sharepoint.com/personal/r_j_janse-5_umcutrecht_nl/Documents/Documenten/GitHub/rjjanse.github.io/publications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="388" documentId="8_{73F58B86-8A8C-44D2-97E6-524D5F699074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD6600C5-4D70-E548-8CE9-1354D7CAD916}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="8_{73F58B86-8A8C-44D2-97E6-524D5F699074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D07A1881-EC02-4849-960E-2C38EC1090E5}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{0D0B8934-B9C8-41E7-88BE-115311452A91}"/>
   </bookViews>
@@ -947,12 +947,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1288,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C16EB68-4490-458C-8DAB-883C12CD690B}">
-  <dimension ref="A1:V32"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" bestFit="1" customWidth="1"/>
@@ -3225,7 +3224,7 @@
         <v>1</v>
       </c>
       <c r="E30">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -3269,9 +3268,6 @@
       <c r="V30" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="M32" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>